<commit_message>
model retrain and test plus dashboard UI changes
</commit_message>
<xml_diff>
--- a/results/metrics_repeated_cv.xlsx
+++ b/results/metrics_repeated_cv.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>f1_score</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
@@ -2725,16 +2737,16 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="B122" t="n">
-        <v>0.836723602484472</v>
+        <v>0.8524242424242423</v>
       </c>
       <c r="C122" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="D122" t="n">
-        <v>0.79995670995671</v>
+        <v>0.8256087050204698</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2744,16 +2756,16 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="B123" t="n">
-        <v>0.9031884057971015</v>
+        <v>0.8629166666666667</v>
       </c>
       <c r="C123" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="D123" t="n">
-        <v>0.8991477272727273</v>
+        <v>0.8358122822299652</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2766,13 +2778,13 @@
         <v>0.875</v>
       </c>
       <c r="B124" t="n">
-        <v>0.8863777089783282</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="C124" t="n">
         <v>0.875</v>
       </c>
       <c r="D124" t="n">
-        <v>0.8752895752895753</v>
+        <v>0.8745173745173744</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2782,16 +2794,16 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="B125" t="n">
-        <v>0.9061919504643964</v>
+        <v>0.8771875000000001</v>
       </c>
       <c r="C125" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="D125" t="n">
-        <v>0.9006250000000001</v>
+        <v>0.8754917387883555</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2801,16 +2813,16 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="B126" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C126" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="D126" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2823,13 +2835,13 @@
         <v>0.875</v>
       </c>
       <c r="B127" t="n">
-        <v>0.8770308123249301</v>
+        <v>0.874927536231884</v>
       </c>
       <c r="C127" t="n">
         <v>0.875</v>
       </c>
       <c r="D127" t="n">
-        <v>0.8754404510218464</v>
+        <v>0.8743727598566308</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -2839,16 +2851,16 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="B128" t="n">
-        <v>0.9181818181818182</v>
+        <v>0.8334821428571428</v>
       </c>
       <c r="C128" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="D128" t="n">
-        <v>0.8991176470588236</v>
+        <v>0.8242307692307692</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2877,16 +2889,16 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>0.925</v>
+        <v>0.9</v>
       </c>
       <c r="B130" t="n">
-        <v>0.9242222222222223</v>
+        <v>0.9125</v>
       </c>
       <c r="C130" t="n">
-        <v>0.925</v>
+        <v>0.9</v>
       </c>
       <c r="D130" t="n">
-        <v>0.9237916219119227</v>
+        <v>0.9007936507936508</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2896,16 +2908,16 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>0.875</v>
+        <v>0.825</v>
       </c>
       <c r="B131" t="n">
-        <v>0.8794117647058822</v>
+        <v>0.8300000000000001</v>
       </c>
       <c r="C131" t="n">
-        <v>0.875</v>
+        <v>0.825</v>
       </c>
       <c r="D131" t="n">
-        <v>0.8755050505050506</v>
+        <v>0.826392961876833</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2915,16 +2927,16 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="B132" t="n">
-        <v>0.9023809523809524</v>
+        <v>0.875</v>
       </c>
       <c r="C132" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="D132" t="n">
-        <v>0.8997782705099778</v>
+        <v>0.875</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -2934,16 +2946,16 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="B133" t="n">
-        <v>0.9</v>
+        <v>0.896875</v>
       </c>
       <c r="C133" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="D133" t="n">
-        <v>0.9</v>
+        <v>0.8720588235294118</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2953,16 +2965,16 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="B134" t="n">
-        <v>0.9</v>
+        <v>0.8767857142857143</v>
       </c>
       <c r="C134" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="D134" t="n">
-        <v>0.9</v>
+        <v>0.8746828752642706</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2972,16 +2984,16 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="B135" t="n">
-        <v>0.7967803030303029</v>
+        <v>0.8569444444444445</v>
       </c>
       <c r="C135" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="D135" t="n">
-        <v>0.7960144927536232</v>
+        <v>0.8125649350649351</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -2991,16 +3003,16 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>0.875</v>
+        <v>0.85</v>
       </c>
       <c r="B136" t="n">
-        <v>0.8839488636363637</v>
+        <v>0.865072463768116</v>
       </c>
       <c r="C136" t="n">
-        <v>0.875</v>
+        <v>0.85</v>
       </c>
       <c r="D136" t="n">
-        <v>0.8742160278745643</v>
+        <v>0.8483193277310924</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3010,16 +3022,16 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>0.825</v>
+        <v>0.75</v>
       </c>
       <c r="B137" t="n">
-        <v>0.830506993006993</v>
+        <v>0.7511446886446886</v>
       </c>
       <c r="C137" t="n">
-        <v>0.825</v>
+        <v>0.75</v>
       </c>
       <c r="D137" t="n">
-        <v>0.8223507148864592</v>
+        <v>0.745748432601881</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3029,16 +3041,16 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>0.85</v>
+        <v>0.875</v>
       </c>
       <c r="B138" t="n">
-        <v>0.85</v>
+        <v>0.8768939393939394</v>
       </c>
       <c r="C138" t="n">
-        <v>0.85</v>
+        <v>0.875</v>
       </c>
       <c r="D138" t="n">
-        <v>0.85</v>
+        <v>0.8753968253968253</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3048,16 +3060,16 @@
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>0.95</v>
+        <v>0.925</v>
       </c>
       <c r="B139" t="n">
-        <v>0.9543478260869565</v>
+        <v>0.9272727272727274</v>
       </c>
       <c r="C139" t="n">
-        <v>0.95</v>
+        <v>0.925</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9495000000000001</v>
+        <v>0.9247357293868921</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3067,16 +3079,16 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>0.875</v>
+        <v>0.85</v>
       </c>
       <c r="B140" t="n">
-        <v>0.8832792207792208</v>
+        <v>0.8640468227424749</v>
       </c>
       <c r="C140" t="n">
-        <v>0.875</v>
+        <v>0.85</v>
       </c>
       <c r="D140" t="n">
-        <v>0.873524783634933</v>
+        <v>0.8471428571428572</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3086,16 +3098,16 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>0.925</v>
+        <v>0.95</v>
       </c>
       <c r="B141" t="n">
-        <v>0.9255952380952381</v>
+        <v>0.9557291666666666</v>
       </c>
       <c r="C141" t="n">
-        <v>0.925</v>
+        <v>0.95</v>
       </c>
       <c r="D141" t="n">
-        <v>0.9246215306980657</v>
+        <v>0.950223799969131</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3105,16 +3117,16 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>0.875</v>
+        <v>0.825</v>
       </c>
       <c r="B142" t="n">
-        <v>0.8777777777777779</v>
+        <v>0.8231481481481481</v>
       </c>
       <c r="C142" t="n">
-        <v>0.875</v>
+        <v>0.825</v>
       </c>
       <c r="D142" t="n">
-        <v>0.8743935309973047</v>
+        <v>0.823361469712016</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3124,16 +3136,16 @@
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>0.875</v>
+        <v>0.9</v>
       </c>
       <c r="B143" t="n">
-        <v>0.8760061919504644</v>
+        <v>0.9135416666666666</v>
       </c>
       <c r="C143" t="n">
-        <v>0.875</v>
+        <v>0.9</v>
       </c>
       <c r="D143" t="n">
-        <v>0.8749034749034749</v>
+        <v>0.9020588235294118</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3165,13 +3177,13 @@
         <v>0.925</v>
       </c>
       <c r="B145" t="n">
-        <v>0.9261609907120743</v>
+        <v>0.9326315789473686</v>
       </c>
       <c r="C145" t="n">
         <v>0.925</v>
       </c>
       <c r="D145" t="n">
-        <v>0.9249420849420849</v>
+        <v>0.9259318141671085</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3181,16 +3193,16 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>0.925</v>
+        <v>0.95</v>
       </c>
       <c r="B146" t="n">
-        <v>0.9284584980237154</v>
+        <v>0.95</v>
       </c>
       <c r="C146" t="n">
-        <v>0.925</v>
+        <v>0.95</v>
       </c>
       <c r="D146" t="n">
-        <v>0.9259878419452887</v>
+        <v>0.95</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3203,13 +3215,13 @@
         <v>0.875</v>
       </c>
       <c r="B147" t="n">
-        <v>0.8748376623376624</v>
+        <v>0.88125</v>
       </c>
       <c r="C147" t="n">
         <v>0.875</v>
       </c>
       <c r="D147" t="n">
-        <v>0.8742983159583</v>
+        <v>0.8722222222222221</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3219,16 +3231,16 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>0.725</v>
+        <v>0.775</v>
       </c>
       <c r="B148" t="n">
-        <v>0.7416666666666666</v>
+        <v>0.8132440476190477</v>
       </c>
       <c r="C148" t="n">
-        <v>0.725</v>
+        <v>0.775</v>
       </c>
       <c r="D148" t="n">
-        <v>0.7213455149501662</v>
+        <v>0.7746010031919744</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3238,16 +3250,16 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>0.975</v>
+        <v>0.9</v>
       </c>
       <c r="B149" t="n">
-        <v>0.9761904761904763</v>
+        <v>0.9033333333333335</v>
       </c>
       <c r="C149" t="n">
-        <v>0.975</v>
+        <v>0.9</v>
       </c>
       <c r="D149" t="n">
-        <v>0.9749016522423289</v>
+        <v>0.9001792114695342</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3257,16 +3269,16 @@
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="B150" t="n">
-        <v>0.919047619047619</v>
+        <v>0.865340909090909</v>
       </c>
       <c r="C150" t="n">
-        <v>0.9</v>
+        <v>0.825</v>
       </c>
       <c r="D150" t="n">
-        <v>0.8997076023391812</v>
+        <v>0.8247683688860159</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3276,16 +3288,16 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>0.875</v>
+        <v>0.8</v>
       </c>
       <c r="B151" t="n">
-        <v>0.8818750000000002</v>
+        <v>0.8066666666666666</v>
       </c>
       <c r="C151" t="n">
-        <v>0.875</v>
+        <v>0.8</v>
       </c>
       <c r="D151" t="n">
-        <v>0.8754200542005419</v>
+        <v>0.8016283524904214</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>

</xml_diff>